<commit_message>
V2.51 out for justins edits
</commit_message>
<xml_diff>
--- a/Manuscript/Manuscript v.2/Supplemental Files (final naming)/Dataset S1. Statistics.xlsx
+++ b/Manuscript/Manuscript v.2/Supplemental Files (final naming)/Dataset S1. Statistics.xlsx
@@ -71,7 +71,7 @@
     <t>Fig1</t>
   </si>
   <si>
-    <t>Fig. 1B–C: behavior, 11-KT, gonadal histology and volume (Table 1)</t>
+    <t>Fig. 1B–C: behavior, 11-KT, gonadal histology and volume</t>
   </si>
   <si>
     <t>FigS1</t>
@@ -128,7 +128,7 @@
     <t>Fig. 6D–F: steroid receptor-associated expression in 6_POA_Mixed</t>
   </si>
   <si>
-    <t>Fig. 1B–C. Behavior, 11-KT, gonadal histology and gonad volume (Table 1)</t>
+    <t>Fig. 1B–C. Behavior, 11-KT, gonadal histology and gonad volume</t>
   </si>
   <si>
     <t>All eight phases. Gonad volume model includes final body length as a covariate.</t>

</xml_diff>